<commit_message>
Implement owner approval message update
</commit_message>
<xml_diff>
--- a/Docs/SmartFlow Beauty Demo.xlsx
+++ b/Docs/SmartFlow Beauty Demo.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="391">
   <si>
     <t>key</t>
   </si>
@@ -367,6 +367,12 @@
     <t>confirmed</t>
   </si>
   <si>
+    <t>req_1781322885424</t>
+  </si>
+  <si>
+    <t>cust_1781322885063</t>
+  </si>
+  <si>
     <t>option_id</t>
   </si>
   <si>
@@ -448,6 +454,9 @@
     <t>opt_1781293783659</t>
   </si>
   <si>
+    <t>opt_1781322885791</t>
+  </si>
+  <si>
     <t>prov_002</t>
   </si>
   <si>
@@ -1087,13 +1096,49 @@
     <t>REQUEST_REJECTED_CLIENT</t>
   </si>
   <si>
-    <t>На жаль, заявку відхилено</t>
-  </si>
-  <si>
-    <t>К сожалению, заявка отклонена</t>
-  </si>
-  <si>
-    <t>Unfortunately, your request was rejected</t>
+    <t>На жаль, заявку відхилено. Ми вам передзвонимо</t>
+  </si>
+  <si>
+    <t>К сожалению, заявка отклонена. Мы Вам перезвоним.</t>
+  </si>
+  <si>
+    <t>Unfortunately, your request was rejected. We will call you back</t>
+  </si>
+  <si>
+    <t>REQUEST_ALREADY_PROCESSED</t>
+  </si>
+  <si>
+    <t>Заявку вже оброблено</t>
+  </si>
+  <si>
+    <t>Заявка уже обработана</t>
+  </si>
+  <si>
+    <t>Request already processed</t>
+  </si>
+  <si>
+    <t>OWNER_REQUEST_CONFIRMED_STATUS</t>
+  </si>
+  <si>
+    <t>✅ Підтверджено</t>
+  </si>
+  <si>
+    <t>✅ Подтверждено</t>
+  </si>
+  <si>
+    <t>✅ Confirmed</t>
+  </si>
+  <si>
+    <t>OWNER_REQUEST_REJECTED_STATUS</t>
+  </si>
+  <si>
+    <t>❌ Відхилено</t>
+  </si>
+  <si>
+    <t>❌ Отклонено</t>
+  </si>
+  <si>
+    <t>❌ Rejected</t>
   </si>
   <si>
     <t>address</t>
@@ -1147,6 +1192,9 @@
     <t>Света</t>
   </si>
   <si>
+    <t>Оля</t>
+  </si>
+  <si>
     <t>start_at</t>
   </si>
   <si>
@@ -1157,6 +1205,9 @@
   </si>
   <si>
     <t>appt_1781293819707</t>
+  </si>
+  <si>
+    <t>appt_1781322908547</t>
   </si>
 </sst>
 </file>
@@ -1214,7 +1265,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1281,6 +1332,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1732,7 +1786,7 @@
         <v>80</v>
       </c>
       <c r="F1" s="17" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="G1" s="17" t="s">
         <v>28</v>
@@ -1749,13 +1803,13 @@
         <v>101</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="F2" s="13">
         <f>+380111111111</f>
@@ -1767,19 +1821,19 @@
     </row>
     <row r="3">
       <c r="A3" s="12" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="F3" s="13">
         <f>+380111111112</f>
@@ -1797,13 +1851,13 @@
         <v>101</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="F4" s="13">
         <f>+380111111113</f>
@@ -1827,19 +1881,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="11" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B1" s="11" t="s">
         <v>66</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="F1" s="11" t="s">
         <v>2</v>
@@ -1847,7 +1901,7 @@
     </row>
     <row r="2">
       <c r="A2" s="12" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>100</v>
@@ -1859,18 +1913,18 @@
         <v>46210.0</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="12" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C3" s="19">
         <v>46188.0</v>
@@ -1879,10 +1933,10 @@
         <v>46188.0</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -1899,19 +1953,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="11" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="F1" s="11" t="s">
         <v>96</v>
@@ -1919,13 +1973,13 @@
     </row>
     <row r="2">
       <c r="A2" s="12" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D2" s="20">
         <v>46187.583333333336</v>
@@ -1937,13 +1991,13 @@
     </row>
     <row r="3">
       <c r="A3" s="12" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D3" s="20">
         <v>46188.5</v>
@@ -1966,9 +2020,9 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="45.13"/>
-    <col customWidth="1" min="2" max="2" width="38.25"/>
+    <col customWidth="1" min="2" max="2" width="40.13"/>
     <col customWidth="1" min="3" max="3" width="49.25"/>
-    <col customWidth="1" min="4" max="4" width="37.13"/>
+    <col customWidth="1" min="4" max="4" width="48.13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1976,657 +2030,699 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>352</v>
+        <v>355</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>367</v>
       </c>
     </row>
   </sheetData>
@@ -2658,10 +2754,10 @@
         <v>80</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>353</v>
+        <v>368</v>
       </c>
       <c r="F1" s="17" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="G1" s="17" t="s">
         <v>85</v>
@@ -2672,16 +2768,16 @@
         <v>101</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>354</v>
+        <v>369</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>354</v>
+        <v>369</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>355</v>
+        <v>370</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>356</v>
+        <v>371</v>
       </c>
       <c r="F2" s="7">
         <f>+380000000001</f>
@@ -2693,19 +2789,19 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>357</v>
+        <v>372</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>359</v>
+        <v>374</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>356</v>
+        <v>371</v>
       </c>
       <c r="F3" s="7">
         <f>+380000000002</f>
@@ -2742,13 +2838,13 @@
         <v>28</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>360</v>
+        <v>375</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>361</v>
+        <v>376</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>97</v>
@@ -2757,10 +2853,10 @@
         <v>30</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>362</v>
+        <v>377</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>363</v>
+        <v>378</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>96</v>
@@ -2768,13 +2864,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>364</v>
+        <v>379</v>
       </c>
       <c r="B2" s="2">
         <v>7.75285374E9</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>365</v>
+        <v>380</v>
       </c>
       <c r="D2" s="7">
         <v>3804562658652</v>
@@ -2794,13 +2890,13 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>366</v>
+        <v>381</v>
       </c>
       <c r="B3" s="2">
         <v>7.75285374E9</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>367</v>
+        <v>382</v>
       </c>
       <c r="D3" s="7">
         <v>38052425635966</v>
@@ -2815,7 +2911,7 @@
         <v>46185.90912765046</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>368</v>
+        <v>383</v>
       </c>
     </row>
     <row r="4">
@@ -2826,7 +2922,7 @@
         <v>7.75285374E9</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D4" s="7">
         <v>3804452125648</v>
@@ -2841,7 +2937,7 @@
         <v>46185.93864143519</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>368</v>
+        <v>383</v>
       </c>
     </row>
     <row r="5">
@@ -2852,7 +2948,7 @@
         <v>7.75285374E9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>369</v>
+        <v>384</v>
       </c>
       <c r="D5" s="7">
         <v>38045245268</v>
@@ -2867,7 +2963,7 @@
         <v>46185.943211805556</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>368</v>
+        <v>383</v>
       </c>
     </row>
     <row r="6">
@@ -2878,7 +2974,7 @@
         <v>7.75285374E9</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D6" s="7">
         <v>3502452635165</v>
@@ -2893,7 +2989,7 @@
         <v>46185.947925671295</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>368</v>
+        <v>383</v>
       </c>
     </row>
     <row r="7">
@@ -2904,7 +3000,7 @@
         <v>7.75285374E9</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D7" s="7">
         <v>38055245256685</v>
@@ -2923,8 +3019,30 @@
       </c>
     </row>
     <row r="8">
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
+      <c r="A8" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B8" s="2">
+        <v>7.75285374E9</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="D8" s="7">
+        <v>3805542545878</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8" s="6">
+        <v>46186.288021562505</v>
+      </c>
+      <c r="G8" s="6">
+        <v>46186.288021562505</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>109</v>
+      </c>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -2944,7 +3062,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="21" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B1" s="21" t="s">
         <v>94</v>
@@ -2962,16 +3080,16 @@
         <v>64</v>
       </c>
       <c r="G1" s="21" t="s">
-        <v>370</v>
+        <v>386</v>
       </c>
       <c r="H1" s="21" t="s">
-        <v>371</v>
+        <v>387</v>
       </c>
       <c r="I1" s="21" t="s">
         <v>96</v>
       </c>
       <c r="J1" s="21" t="s">
-        <v>372</v>
+        <v>388</v>
       </c>
       <c r="K1" s="17" t="s">
         <v>97</v>
@@ -2982,7 +3100,7 @@
     </row>
     <row r="2">
       <c r="A2" s="18" t="s">
-        <v>373</v>
+        <v>389</v>
       </c>
       <c r="B2" s="18" t="s">
         <v>62</v>
@@ -3012,6 +3130,38 @@
       </c>
       <c r="L2" s="6">
         <v>46185.95161697917</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="G3" s="23">
+        <v>46187.395833333336</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="K3" s="6">
+        <v>46186.28829336805</v>
+      </c>
+      <c r="L3" s="6">
+        <v>46186.28829336805</v>
       </c>
     </row>
   </sheetData>
@@ -3047,7 +3197,7 @@
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="6">
-        <v>46185.951275659725</v>
+        <v>46186.28811368055</v>
       </c>
     </row>
     <row r="3">
@@ -4223,6 +4373,29 @@
         <v>46185.95118355324</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="G6" s="6">
+        <v>46186.28802574074</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -4241,19 +4414,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>94</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>96</v>
@@ -4264,10 +4437,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C2" s="10">
         <v>46186.0</v>
@@ -4287,10 +4460,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C3" s="10">
         <v>46185.0</v>
@@ -4310,10 +4483,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C4" s="10">
         <v>46186.0</v>
@@ -4333,10 +4506,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C5" s="10">
         <v>46187.0</v>
@@ -4356,10 +4529,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>118</v>
       </c>
       <c r="C6" s="10">
         <v>46185.0</v>
@@ -4379,10 +4552,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C7" s="10">
         <v>46186.0</v>
@@ -4402,10 +4575,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C8" s="10">
         <v>46187.0</v>
@@ -4425,10 +4598,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>124</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>122</v>
       </c>
       <c r="C9" s="10">
         <v>46185.0</v>
@@ -4448,10 +4621,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C10" s="10">
         <v>46186.0</v>
@@ -4471,10 +4644,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C11" s="10">
         <v>46186.0</v>
@@ -4494,10 +4667,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C12" s="10">
         <v>46186.0</v>
@@ -4517,10 +4690,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C13" s="10">
         <v>46186.0</v>
@@ -4532,7 +4705,7 @@
         <v>1.0</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G13" s="6">
         <v>46185.90712123843</v>
@@ -4540,10 +4713,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C14" s="10">
         <v>46185.0</v>
@@ -4555,7 +4728,7 @@
         <v>1.0</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G14" s="6">
         <v>46185.909134305555</v>
@@ -4563,7 +4736,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>62</v>
@@ -4578,10 +4751,33 @@
         <v>1.0</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G15" s="6">
         <v>46185.95119975695</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C16" s="10">
+        <v>46187.0</v>
+      </c>
+      <c r="D16" s="15">
+        <v>0.3958333333321207</v>
+      </c>
+      <c r="E16" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="G16" s="6">
+        <v>46186.28802998843</v>
       </c>
     </row>
   </sheetData>
@@ -4631,7 +4827,7 @@
     </row>
     <row r="4">
       <c r="A4" s="12" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>86</v>
@@ -4657,13 +4853,13 @@
         <v>66</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="E1" s="11" t="s">
         <v>85</v>
@@ -4674,7 +4870,7 @@
         <v>100</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C2" s="16">
         <v>0.375</v>
@@ -4691,7 +4887,7 @@
         <v>100</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C3" s="16">
         <v>0.4166666666666667</v>

</xml_diff>